<commit_message>
DE feed v2: no parents, TTX-based ingredients/weights, texts for all missing positions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDVF22cVHqURRrq6mrUjqS
</commit_message>
<xml_diff>
--- a/DE_Feed_Missing_Positions/DE_SEO_Texte_Missing_Positions.xlsx
+++ b/DE_Feed_Missing_Positions/DE_SEO_Texte_Missing_Positions.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DE Texte - im Feed" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DE Texte - weitere Positionen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benötigte Templates" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1385,12 +1386,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Не включён: Inactive на UK</t>
+          <t>Тексты готовы, Inactive на UK</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Листинг на UK неактивен, решение нужно от владельца</t>
+          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
         </is>
       </c>
     </row>
@@ -1428,12 +1429,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Не включён: Inactive на UK</t>
+          <t>Тексты готовы, Inactive на UK</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Листинг на UK неактивен, решение нужно от владельца</t>
+          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1472,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Не включён: Inactive на UK</t>
+          <t>Тексты готовы, Inactive на UK</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Листинг на UK неактивен, решение нужно от владельца</t>
+          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1515,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Не включён: Inactive на UK</t>
+          <t>Тексты готовы, Inactive на UK</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Листинг на UK неактивен, решение нужно от владельца</t>
+          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
         </is>
       </c>
     </row>
@@ -1534,600 +1535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="80" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="50" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Item Name (≤75)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Zeichen</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Item Highlight (≤125)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Zeichen</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Bullet 1</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Bullet 2</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Bullet 3</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Bullet 4</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Bullet 5</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Max Bullet</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Description (≤2000)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Zeichen</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Search Terms (≤249 Byte)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Byte</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>DE-Parent-3</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Körperlotion 125 ml, tägliche Feuchtigkeitspflege</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Kamelmilch oder Ziegenmilch, leicht einziehend, nicht fettend, zwei Varianten</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Zwei Varianten: Zwei Körperlotionen in einer Serie, jede in der 125-ml-Flasche, wählen Sie nach Milchsorte: Kamelmilch oder Ziegenmilch</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Gleiche Textur: Gleiche leichte, schnell einziehende Textur für alle Varianten, zur täglichen Pflege von Körper und Händen</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Anwendung: Auf die gereinigte Haut auftragen, am besten nach dem Duschen, Inhaltsstoffe und Hauttyp siehe Variante</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="n">
-        <v>135</v>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Die ZAptieka Körperlotion gibt es als Serie mit zwei 125-ml-Varianten, die sich durch die Milchsorte unterscheiden: Kamelmilch oder Ziegenmilch. Beide Lotionen sind leicht, ziehen schnell ein und hinterlassen keinen fettigen Film. Wählen Sie eine Variante, um die vollständige Beschreibung, die Inhaltsstoffe und die Anwendung zu sehen.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>336</v>
-      </c>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>TG-5RTH-70GN</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Moringa Gesichtscreme 60 ml für Damen und Herren</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Mit Sheabutter, Jojoba- und Weizenkeimöl, Tag und Nacht, für normale, trockene und Mischhaut</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Moringaöl: Aus den Samen des Moringabaums, von Natur aus reich an Fettsäuren und für sein leichtes Einziehen in der Hautpflege geschätzt</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Leichte Textur: Zieht ohne Fettfilm ein, trägt sich angenehm tagsüber und unter Make-up und ist reichhaltig genug für den Abend</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Sheabutter: Sorgt für anhaltende Pflege, damit sich die Haut auch Stunden später noch weich anfühlt und nicht spannt</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Für jeden Tag: Feuchtigkeitscreme für Gesicht und Hals, morgens und abends, für normale, trockene und Mischhaut, für Damen und Herren</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Ergiebig: Eine erbsengroße Menge reicht für Gesicht und Hals, deshalb hält der 60-ml-Tiegel lange</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>136</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Moringa ist der Inhaltsstoff dieser Pflegeserie, den die wenigsten schon ausprobiert haben. Das Öl wird aus den Samen des Moringabaums gepresst und ist von Natur aus reich an Fettsäuren, zieht aber deutlich leichter ein als schwerere Pflanzenöle.
-Genau das prägt diese Gesichtscreme: Sie legt sich leicht auf die Haut, zieht ohne Film ein und lässt sich tagsüber und unter Make-up gut tragen. Die Sheabutter in der Basis sorgt dafür, dass sich die Haut auch Stunden später noch weich anfühlt und nicht schon mittags spannt.
-Die Creme ist als Feuchtigkeitscreme für jeden Tag gedacht, nicht als aufwendige Kur. Sie eignet sich für normale, trockene und Mischhaut, für Damen und Herren.
-Anwendung: Morgens und abends auf die gereinigte Haut auftragen. Eine kleine Menge zwischen den Fingerspitzen erwärmen und mit sanften Streichbewegungen nach oben in Gesicht und Hals einarbeiten. Vor dem Make-up eine Minute einziehen lassen.
-Wichtige Inhaltsstoffe: Moringasamenöl, Sheabutter, Jojobasamenöl, Olivenöl, Weizenkeimöl, Bienenwachs, Glycerin, Allantoin, Vitamin E. Inhalt: 60 ml, Tiegel 5,5 x 5 cm.
-Nur zur äußerlichen Anwendung. Bei empfindlicher Haut vor der ersten Anwendung an einer kleinen Stelle testen.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>1212</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>tagescreme nachtcreme pflegecreme gesichtspflege unisex naturkosmetik bodybutter handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend sensitive geschenkidee weihnachtsgeschenk muttertag vegan</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>F8-4Y8G-GT5L</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Kamelmilch Körperlotion 125 ml für Körper und Gesicht</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Mit Olivenöl, Glycerin und Panthenol, leicht einziehend, nicht fettend, für trockene und normale Haut</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>101</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Kamelmilch: In der Hautpflege des Nahen Ostens seit Generationen geschätzt, bringt von Natur aus Proteine, Aminosäuren und Vitamine in die tägliche Lotion</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Zieht schnell ein: Die leichte Textur hinterlässt keinen klebrigen Film, Sie können sich direkt nach dem Eincremen anziehen</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Glycerin und Panthenol: Zwei bewährte Feuchtigkeitsspender, die Wasser in der Haut halten, damit sie sich auch Stunden später angenehm anfühlt</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Nach der Dusche: Auf leicht feuchter Haut bindet die Lotion am meisten Feuchtigkeit, auch angenehm nach einem Tag im Freien</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Für Körper und Gesicht: Leicht genug fürs Gesicht, ergiebig für Arme, Beine und Hände, alles in einer 125-ml-Flasche</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>154</v>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Kamelmilch klingt exotisch und erweist sich als ausgesprochen praktisch. Sie wird in der Hautpflege des Nahen Ostens seit Generationen verwendet und enthält von Natur aus Proteine, Aminosäuren, Milchfette und Vitamine. Das passt zu einer Lotion, die jeden Tag benutzt wird.
-Die Rezeptur verbindet Kamelmilch mit Glycerin und Panthenol, zwei zuverlässigen Feuchtigkeitsspendern, die Wasser in der Haut halten. Deshalb fühlt sich die Haut auch Stunden nach dem Auftragen noch angenehm an. Olivenöl rundet die Lotion ab und pflegt, ohne die Textur schwer zu machen.
-Bei einer Körperlotion zählt vor allem das Einziehen: Diese Lotion ist bewusst leicht, lässt sich gut verteilen, zieht schnell ein und klebt nicht. Dadurch eignet sie sich auch fürs Gesicht, was bei einer dicken Körpercreme selten möglich ist.
-Anwendung: Auf die gereinigte Haut auftragen, am besten direkt nach dem Duschen, solange die Haut noch leicht feucht ist. In Arme, Beine, Hände und Körper einmassieren, für Gesicht und Hals eine kleinere Menge verwenden.
-Inhalt: 125 ml, Flasche 12,5 x 4 cm. Wichtige Inhaltsstoffe: Kamelmilch (Camelus Lactis), Olivenöl, Glycerin, Panthenol. Für trockene und normale Haut, für Damen und Herren. Nur zur äußerlichen Anwendung.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>1236</v>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>bodylotion körpermilch bodymilch feuchtigkeitslotion handlotion duschen pflegelotion damen herren unisex naturkosmetik bodybutter handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend sensitive geschenkidee weihnachtsgeschenk</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>UX-E5I6-5O5L</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Ziegenmilch Körperlotion 125 ml, trockene empfindliche Haut</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Leichte Tageslotion mit pflegenden Ölen, zieht schnell ein, nicht fettend, für Damen und Herren</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Ziegenmilch: Der Klassiker für Haut, die auf gewöhnliche Lotionen reagiert, mit von Natur aus enthaltenen Milchfetten, Vitaminen und Mineralstoffen</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Für trockene und empfindliche Haut: Sanfte Rezeptur für raue, spannende Haut, auch für alle, die stark parfümierte Lotionen nicht vertragen</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Leichte Textur: Zieht schnell ein und hinterlässt keinen fettigen Rückstand, Sie können sich direkt danach anziehen</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Auf feuchter Haut: Wenige Minuten nach dem Duschen aufgetragen, solange die Haut noch leicht feucht ist, bindet die Lotion am meisten Feuchtigkeit</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Für jeden Tag: 125 ml genug für die regelmäßige Pflege von Armen, Beinen, Ellbogen und Knien statt einer winzigen Probiergröße</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>147</v>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Ziegenmilch wird seit Jahrhunderten in der Hautpflege verwendet, und ihr Ruf beruht auf Milde. Sie enthält von Natur aus Milchfette, Proteine, Vitamine und Mineralstoffe, und Lotionen auf dieser Basis vertragen oft auch Menschen, deren Haut auf Standardprodukte aus dem Drogeriemarkt reagiert.
-Diese Körperlotion für trockene und empfindliche Haut ist bewusst leicht gehalten. Eine dicke, fettige Body Butter bleibt oft ungenutzt im Schrank, eine Lotion, die in Sekunden einzieht, wird dagegen täglich benutzt. Und bei der Hautpflege zählt die Regelmäßigkeit mehr als die Reichhaltigkeit.
-Pflegende Pflanzenöle in der Basis sorgen dafür, dass sich die Haut weich anfühlt und nicht nur beschichtet. Auf schweren Duft wurde bewusst verzichtet, das ist für reaktive Haut sinnvoll.
-Anwendung: Täglich auf die gereinigte Haut auftragen, am besten nach dem Duschen oder Baden. In Arme, Beine, Körper und Hände einmassieren, bis die Lotion eingezogen ist. Besonders trockene Stellen wie Ellbogen, Knie und Schienbeine bei Bedarf erneut eincremen.
-Inhalt: 125 ml, Flasche 12,5 x 4 cm. Wichtige Inhaltsstoffe: Ziegenmilch (Caprae Lac), Olivenöl, Glycerin, Panthenol. Für trockene, empfindliche und normale Haut, für Damen und Herren. Nur zur äußerlichen Anwendung. Bei empfindlicher Haut vor der ersten Anwendung testen.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>1315</v>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>bodylotion körpermilch bodymilch hautpflege feuchtigkeitslotion sensitive pflegelotion tägliche knie unisex naturkosmetik hautverträglich bodybutter handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend geschenkidee muttertag</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="n">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>DP-ZW1J-GZYS</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Körpercreme 60 ml mit Sheabutter und Geranie</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Mit Jojoba- und Olivenöl, für Gesicht und Körper, Tag und Nacht, für trockene und normale Haut</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>94</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Geranie: Das ätherische Geranienöl hat einen weichen, grünen Blütenduft, damit duftet die Creme nach etwas und nicht nach Apotheke</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Für Gesicht und Körper: Reichhaltig genug für trockene Stellen am Körper, leicht genug fürs Gesicht, ein Tiegel ersetzt zwei Produkte</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Sheabutter und Pflanzenöle: Sheabutter, Jojoba- und Olivenöl bilden die Basis und pflegen die Haut, statt nur an der Oberfläche zu liegen</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Geschmeidig den ganzen Tag: Für Haut, die nach dem Waschen, bei Kälte oder in trockener Heizungsluft spannt und mit einer leichten Lotion nicht auskommt</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Morgens und abends: Zieht gut genug für tagsüber ein und ist reichhaltig genug für den Abend, für Damen und Herren</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>152</v>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Geranie gehört zu den unterschätzten ätherischen Ölen. Sie duftet weich, grün und blumig, weniger süß als Rose und weniger scharf als Zitrus. Deshalb riecht diese Creme nach etwas, das man sich aussuchen würde, und nicht nach Medizin.
-Unter dem Duft steckt eine echte Feuchtigkeitspflege für trockene Haut. Sheabutter bildet die Basis und gibt der Creme ihre Substanz, Jojoba- und Olivenöl pflegen die Haut, während sie Feuchtigkeit spenden. Die Mischung richtet sich an Haut, die nach dem Waschen spannt und unter einer leichten Lotion nicht lange angenehm bleibt.
-Die Textur ist reichhaltig genug für den Körper, etwa für trockene Stellen an Ellbogen, Knien und Schienbeinen, zieht aber im Gesicht ohne fettigen Film ein. So kann ein Tiegel Gesichtscreme und Körpercreme ersetzen, was auch auf Reisen praktisch ist.
-Anwendung: Morgens und abends auf die gereinigte Haut auftragen. Eine kleine Menge zwischen den Fingern erwärmen und in Gesicht und Hals einarbeiten, an trockenen Körperstellen großzügiger auftragen, am besten direkt nach dem Duschen auf noch leicht feuchter Haut.
-Für trockene und normale Haut, für Damen und Herren. Nur zur äußerlichen Anwendung. Die Creme enthält ätherisches Geranienöl, bei empfindlicher Haut vor der ersten Anwendung testen.
-Inhalt: 60 ml, Tiegel 5,5 x 5 cm. Wichtige Inhaltsstoffe: Sheabutter, Geranienöl, Jojobasamenöl, Olivenöl, Weizenkeimöl, Bienenwachs, Glycerin, Allantoin, Vitamin E.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>1435</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>bodycream bodybutter gesichtscreme hautpflege feuchtigkeitscreme tagescreme nachtcreme ellbogen reisegröße pflegecreme naturkosmetik handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend sensitive geschenkidee muttertag vegan</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>BF-UJUW-N586</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Rosmarin Haaröl 100 ml mit Rizinusöl und Arganöl</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Ohne Wasser und Silikon, mit Rucolasamen-, Weizenkeim- und Zitronengrasöl, für Kopfhaut und Haarlängen</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>102</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Sechs Öle, kein Wasser, kein Silikon: Rizinus-, Rucolasamen-, Weizenkeim- und Arganöl mit ätherischem Rosmarin- und Zitronengrasöl, Sie tragen die reine Ölmischung auf</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Rizinusöl als Basis: Das dickflüssige, klassische Kopfhautöl wird seit Generationen in die Haarwurzeln einmassiert und umhüllt das Haar besser als ein dünnes Öl allein</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Rosmarin und Argan: Rosmarinöl gibt der Mischung den frischen, kräuterigen Duft, Arganöl glättet die Schuppenschicht, damit die Längen glänzen statt nur ölig zu wirken</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Kopfhautmassage: Zwei bis drei Minuten mit den Fingerspitzen einmassieren, so wird die Anwendung zur Routine, die man gern beibehält</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Auch für die Längen: Ein bis zwei Tropfen zwischen den Handflächen verreiben und in trockene Spitzen streichen, so deckt eine Flasche Kopfhautpflege und Finish ab</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>167</v>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Ein Kopfhaut- und Haaröl aus sechs Ölen und sonst nichts. Es enthält weder Wasser noch Silikon: Auf die Kopfhaut kommt keine verdünnte Lotion, sondern die Ölmischung selbst.
-Rizinusöl bildet die Basis. Es ist das dickflüssige, traditionelle Kopfhautöl, das seit Generationen in die Haarwurzeln einmassiert wird, und es gibt der Mischung genug Substanz, um den Haarschaft zu umhüllen, statt zu verdunsten. Rucolasamenöl und Weizenkeimöl ergänzen es, und Arganöl glättet die Schuppenschicht, sodass das Haar glänzend aussieht.
-Die beiden ätherischen Öle sind Rosmarin und Zitronengras. Rosmarin gibt der Mischung den frischen, kräuterigen Duft, Zitronengras macht ihn spritziger, damit das Öl nicht schwer riecht.
-Anwendung: Das Haar in Partien teilen, entlang jedes Scheitels einige Tropfen auftragen und zwei bis drei Minuten in die Kopfhaut einmassieren. Mindestens eine Stunde einwirken lassen, auf Wunsch auch über Nacht, danach mit Shampoo auswaschen. Für die Längen ein bis zwei Tropfen zwischen den Handflächen verreiben und über trockene Spitzen streichen. Üblich sind ein- bis zweimal pro Woche.
-Geeignet für alle Haartypen, für Damen und Herren. Inhalt: 100 ml, Flasche 13,5 x 4 cm. Inhaltsstoffe: Ricinus Communis Seed Oil, Eruca Sativa Seed Oil, Triticum Vulgare Germ Oil, Argania Spinosa Kernel Oil, Rosmarinus Officinalis Leaf Oil, Cymbopogon Citratus Oil. Nur zur äußerlichen Anwendung, von Kindern fernhalten.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>1428</v>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>haarpflege haarserum haarkur haarwuchs haarwachstum pflegeöl ölkur vor haarwäsche spliss damen herren unisex pipette naturkosmetik haarmaske haarbehandlung trockenes geschenk haarpflegeset pflanzenöl</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>YJ-OPSZ-IOCI</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>ZAptieka Rosmarin Haarspülung 250 ml mit Argan- und Jojobaöl</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Sulfatfrei, ohne Silikone, Parabene und Mineralöl, mit Weizenkeimöl und Panthenol, entwirrt, für alle Haartypen</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>111</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Rosmarin: Der Pflegestoff, nach dem viele suchen, steckt hier in dem Schritt, den Sie nach jeder Haarwäsche ohnehin machen</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Jojoba-, Argan- und Weizenkeimöl: Drei pflegende Pflanzenöle statt Silikon, damit sich das Haar wirklich weicher anfühlt und nicht nur kurz beschichtet</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Leichteres Kämmen: Die Spülung lässt den Kamm durch das nasse Haar gleiten, ohne Ziehen, das an den Spitzen zu Haarbruch führen kann</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Für alle Haartypen: Beschwert feines Haar nicht und pflegt trockene, dicke oder krause Längen, für Damen und Herren, für die ganze Familie</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Passend zum Shampoo: Als Duo mit dem ZAptieka Rosmarin Shampoo konzipiert, funktioniert aber auch mit jedem anderen Shampoo</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>151</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Rosmarin ist zum meistbeachteten Inhaltsstoff der Haarpflege geworden, doch die Aufmerksamkeit gilt meist Ölen und Seren. Die Haarspülung wird dabei übersehen, obwohl sie der Schritt ist, den Sie nach jeder einzelnen Haarwäsche verwenden.
-Diese Spülung basiert auf Rosmarin und drei pflegenden Pflanzenölen: Jojoba-, Argan- und Weizenkeimöl. Das ist wichtiger, als es klingt. Viele Spülungen setzen auf Silikone für das Gleitgefühl, das Haar fühlt sich sofort glatt an und nach einer Woche beschichtet. Pflanzenöle pflegen das Haar selbst, sodass die Weichheit auch nach mehreren Haarwäschen bleibt.
-Die Haarspülung ist sulfatfrei und silikonfrei: Sie enthält keine Sulfattenside und keine Silikone, die die Pflege ersetzen.
-Der praktische Vorteil ist das Entwirren. Nach der Wäsche ist das Haar am empfindlichsten, und das Durchziehen des Kamms durch Knoten ist eine häufige Ursache für Haarbruch an den Spitzen. Lässt sich der Kamm frei bewegen, schützt das die Längen über Monate.
-Die Spülung ist für alle Haartypen ausgewogen, für Damen und Herren. Feines Haar wird nicht beschwert, trockene, dicke oder krause Längen werden ausreichend gepflegt. Sie hinterlässt außerdem den kräuterigen Rosmarinduft.
-Anwendung: Nach dem Shampoonieren überschüssiges Wasser ausdrücken, von den Längen bis in die Spitzen auftragen und die Haaransätze aussparen, wenn Ihr Haar schnell fettet. Zwei bis drei Minuten einwirken lassen, durchkämmen und gründlich ausspülen.
-Inhalt: 250 ml, Flasche 19 x 5 cm. Wichtige Inhaltsstoffe: Cetearylalkohol, Jojobasamenöl, Weizenkeimöl, Arganöl, Rosmarinblattöl, Panthenol, Glycerin. Frei von Sulfaten, SLS, SLES, Parabenen, Silikonen und Mineralöl. Nur zur äußerlichen Anwendung.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>1710</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>conditioner haarkur pflegespülung haarpflege kopfhaut trockenes strapaziertes entwirren kämmbarkeit glanz weich naturkosmetik unisex haarmaske haarbehandlung kopfhautpflege geschenk haarpflegeset rosmarinöl pflanzenöl</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>221</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2146,6 +1554,7 @@
     <col width="50" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2226,6 +1635,615 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Inhaltsstoffe INCI (TTX)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Gewicht g (TTX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TG-5RTH-70GN</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Moringa Gesichtscreme 60 ml für Damen und Herren</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Mit Sheabutter, Jojoba- und Weizenkeimöl, Tag und Nacht, für normale, trockene und Mischhaut</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Moringaöl: Aus den Samen des Moringabaums, von Natur aus reich an Fettsäuren und für sein leichtes Einziehen in der Hautpflege geschätzt</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Leichte Textur: Zieht ohne Fettfilm ein, trägt sich angenehm tagsüber und unter Make-up und ist reichhaltig genug für den Abend</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sheabutter: Sorgt für anhaltende Pflege, damit sich die Haut auch Stunden später noch weich anfühlt und nicht spannt</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Für jeden Tag: Feuchtigkeitscreme für Gesicht und Hals, morgens und abends, für normale, trockene und Mischhaut, für Damen und Herren</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Ergiebig: Eine erbsengroße Menge reicht für Gesicht und Hals, deshalb hält der 60-ml-Tiegel lange</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Moringa ist der Inhaltsstoff dieser Pflegeserie, den die wenigsten schon ausprobiert haben. Das Öl wird aus den Samen des Moringabaums gepresst und ist von Natur aus reich an Fettsäuren, zieht aber deutlich leichter ein als schwerere Pflanzenöle.
+Genau das prägt diese Gesichtscreme: Sie legt sich leicht auf die Haut, zieht ohne Film ein und lässt sich tagsüber und unter Make-up gut tragen. Die Sheabutter in der Basis sorgt dafür, dass sich die Haut auch Stunden später noch weich anfühlt und nicht schon mittags spannt.
+Die Creme ist als Feuchtigkeitscreme für jeden Tag gedacht, nicht als aufwendige Kur. Sie eignet sich für normale, trockene und Mischhaut, für Damen und Herren.
+Anwendung: Morgens und abends auf die gereinigte Haut auftragen. Eine kleine Menge zwischen den Fingerspitzen erwärmen und mit sanften Streichbewegungen nach oben in Gesicht und Hals einarbeiten. Vor dem Make-up eine Minute einziehen lassen.
+Inhaltsstoffe (INCI): Aqua, Stearic Acid, Cetyl Alcohol, Simmondsia Chinensis Seed Oil, Isopropyl Myristate, Triethanolamine, Phenoxyethanol, BHT, Moringa Oleifera Seed Oil, Allantoin, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Glycerin, Cera Alba, Tocopheryl Acetate, Triticum Vulgare Germ Oil. Inhalt: 60 ml, Tiegel 5,5 x 5 cm.
+Nur zur äußerlichen Anwendung. Bei empfindlicher Haut vor der ersten Anwendung an einer kleinen Stelle testen. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>1405</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>tagescreme nachtcreme pflegecreme gesichtspflege unisex naturkosmetik bodybutter handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend sensitive geschenkidee weihnachtsgeschenk muttertag vegan</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>209</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Aqua, Stearic Acid, Cetyl Alcohol, Simmondsia Chinensis Seed Oil, Isopropyl Myristate, Triethanolamine, Phenoxyethanol, BHT, Moringa Oleifera Seed Oil, Allantoin, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Glycerin, Cera Alba, Tocopheryl Acetate, Triticum Vulgare Germ Oil</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>F8-4Y8G-GT5L</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Kamelmilch Körperlotion 125 ml für Körper und Gesicht</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Mit Olivenöl, Glycerin und Panthenol, leicht einziehend, nicht fettend, für trockene und normale Haut</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Kamelmilch: In der Hautpflege des Nahen Ostens seit Generationen geschätzt, bringt von Natur aus Proteine, Aminosäuren und Vitamine in die tägliche Lotion</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Zieht schnell ein: Die leichte Textur hinterlässt keinen klebrigen Film, Sie können sich direkt nach dem Eincremen anziehen</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Glycerin und Panthenol: Zwei bewährte Feuchtigkeitsspender, die Wasser in der Haut halten, damit sie sich auch Stunden später angenehm anfühlt</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Nach der Dusche: Auf leicht feuchter Haut bindet die Lotion am meisten Feuchtigkeit, auch angenehm nach einem Tag im Freien</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Für Körper und Gesicht: Leicht genug fürs Gesicht, ergiebig für Arme, Beine und Hände, alles in einer 125-ml-Flasche</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>154</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Kamelmilch klingt exotisch und erweist sich als ausgesprochen praktisch. Sie wird in der Hautpflege des Nahen Ostens seit Generationen verwendet und enthält von Natur aus Proteine, Aminosäuren, Milchfette und Vitamine. Das passt zu einer Lotion, die jeden Tag benutzt wird.
+Die Rezeptur verbindet Kamelmilch mit Glycerin und Panthenol, zwei zuverlässigen Feuchtigkeitsspendern, die Wasser in der Haut halten. Deshalb fühlt sich die Haut auch Stunden nach dem Auftragen noch angenehm an. Olivenöl rundet die Lotion ab und pflegt, ohne die Textur schwer zu machen.
+Bei einer Körperlotion zählt vor allem das Einziehen: Diese Lotion ist bewusst leicht, lässt sich gut verteilen, zieht schnell ein und klebt nicht. Dadurch eignet sie sich auch fürs Gesicht, was bei einer dicken Körpercreme selten möglich ist.
+Anwendung: Auf die gereinigte Haut auftragen, am besten direkt nach dem Duschen, solange die Haut noch leicht feucht ist. In Arme, Beine, Hände und Körper einmassieren, für Gesicht und Hals eine kleinere Menge verwenden.
+Inhalt: 125 ml, Flasche 12,5 x 4 cm. Inhaltsstoffe (INCI): Aqua, Olea Europaea (Olive) Fruit Oil, Glycerin, Isopropyl Myristate, Cetearyl Alcohol, Glyceryl Stearate, PEG-40 Hydrogenated Castor Oil, Panthenol, Camelus Lactis, Phenoxyethanol. Für trockene und normale Haut, für Damen und Herren. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>1378</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>bodylotion körpermilch bodymilch feuchtigkeitslotion handlotion duschen pflegelotion damen herren unisex naturkosmetik bodybutter handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend sensitive geschenkidee weihnachtsgeschenk</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>243</v>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Aqua, Olea Europaea (Olive) Fruit Oil, Glycerin, Isopropyl Myristate, Cetearyl Alcohol, Glyceryl Stearate, PEG-40 Hydrogenated Castor Oil, Panthenol, Camelus Lactis, Phenoxyethanol</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>UX-E5I6-5O5L</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Ziegenmilch Körperlotion 125 ml, trockene empfindliche Haut</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Leichte Tageslotion mit pflegenden Ölen, zieht schnell ein, nicht fettend, für Damen und Herren</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Ziegenmilch: Der Klassiker für Haut, die auf gewöhnliche Lotionen reagiert, mit von Natur aus enthaltenen Milchfetten, Vitaminen und Mineralstoffen</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Für trockene und empfindliche Haut: Sanfte Rezeptur für raue, spannende Haut, auch für alle, die stark parfümierte Lotionen nicht vertragen</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Leichte Textur: Zieht schnell ein und hinterlässt keinen fettigen Rückstand, Sie können sich direkt danach anziehen</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Auf feuchter Haut: Wenige Minuten nach dem Duschen aufgetragen, solange die Haut noch leicht feucht ist, bindet die Lotion am meisten Feuchtigkeit</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Für jeden Tag: 125 ml genug für die regelmäßige Pflege von Armen, Beinen, Ellbogen und Knien statt einer winzigen Probiergröße</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Ziegenmilch wird seit Jahrhunderten in der Hautpflege verwendet, und ihr Ruf beruht auf Milde. Sie enthält von Natur aus Milchfette, Proteine, Vitamine und Mineralstoffe, und Lotionen auf dieser Basis vertragen oft auch Menschen, deren Haut auf Standardprodukte aus dem Drogeriemarkt reagiert.
+Diese Körperlotion für trockene und empfindliche Haut ist bewusst leicht gehalten. Eine dicke, fettige Body Butter bleibt oft ungenutzt im Schrank, eine Lotion, die in Sekunden einzieht, wird dagegen täglich benutzt. Und bei der Hautpflege zählt die Regelmäßigkeit mehr als die Reichhaltigkeit.
+Pflegende Pflanzenöle in der Basis sorgen dafür, dass sich die Haut weich anfühlt und nicht nur beschichtet. Auf schweren Duft wurde bewusst verzichtet, das ist für reaktive Haut sinnvoll.
+Anwendung: Täglich auf die gereinigte Haut auftragen, am besten nach dem Duschen oder Baden. In Arme, Beine, Körper und Hände einmassieren, bis die Lotion eingezogen ist. Besonders trockene Stellen wie Ellbogen, Knie und Schienbeine bei Bedarf erneut eincremen.
+Inhalt: 125 ml, Flasche 12,5 x 4 cm. Inhaltsstoffe (INCI): Aqua, Olea Europaea (Olive) Fruit Oil, Glycerin, Isopropyl Myristate, Cetearyl Alcohol, Glyceryl Stearate, PEG-40 Hydrogenated Castor Oil, Panthenol, Caprae Lac, Phenoxyethanol. Für trockene, empfindliche und normale Haut, für Damen und Herren. Nur zur äußerlichen Anwendung. Bei empfindlicher Haut vor der ersten Anwendung testen. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>1456</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>bodylotion körpermilch bodymilch hautpflege feuchtigkeitslotion sensitive pflegelotion tägliche knie unisex naturkosmetik hautverträglich bodybutter handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend geschenkidee muttertag</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>245</v>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Aqua, Olea Europaea (Olive) Fruit Oil, Glycerin, Isopropyl Myristate, Cetearyl Alcohol, Glyceryl Stearate, PEG-40 Hydrogenated Castor Oil, Panthenol, Caprae Lac, Phenoxyethanol</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>DP-ZW1J-GZYS</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Körpercreme 60 ml mit Sheabutter und Geranie</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Mit Jojoba- und Olivenöl, für Gesicht und Körper, Tag und Nacht, für trockene und normale Haut</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Geranie: Das ätherische Geranienöl hat einen weichen, grünen Blütenduft, damit duftet die Creme nach etwas und nicht nach Apotheke</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Für Gesicht und Körper: Reichhaltig genug für trockene Stellen am Körper, leicht genug fürs Gesicht, ein Tiegel ersetzt zwei Produkte</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Sheabutter und Pflanzenöle: Sheabutter, Jojoba- und Olivenöl bilden die Basis und pflegen die Haut, statt nur an der Oberfläche zu liegen</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Geschmeidig den ganzen Tag: Für Haut, die nach dem Waschen, bei Kälte oder in trockener Heizungsluft spannt und mit einer leichten Lotion nicht auskommt</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Morgens und abends: Zieht gut genug für tagsüber ein und ist reichhaltig genug für den Abend, für Damen und Herren</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>152</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Geranie gehört zu den unterschätzten ätherischen Ölen. Sie duftet weich, grün und blumig, weniger süß als Rose und weniger scharf als Zitrus. Deshalb riecht diese Creme nach etwas, das man sich aussuchen würde, und nicht nach Medizin.
+Unter dem Duft steckt eine echte Feuchtigkeitspflege für trockene Haut. Sheabutter bildet die Basis und gibt der Creme ihre Substanz, Jojoba- und Olivenöl pflegen die Haut, während sie Feuchtigkeit spenden. Die Mischung richtet sich an Haut, die nach dem Waschen spannt und unter einer leichten Lotion nicht lange angenehm bleibt.
+Die Textur ist reichhaltig genug für den Körper, etwa für trockene Stellen an Ellbogen, Knien und Schienbeinen, zieht aber im Gesicht ohne fettigen Film ein. So kann ein Tiegel Gesichtscreme und Körpercreme ersetzen, was auch auf Reisen praktisch ist.
+Anwendung: Morgens und abends auf die gereinigte Haut auftragen. Eine kleine Menge zwischen den Fingern erwärmen und in Gesicht und Hals einarbeiten, an trockenen Körperstellen großzügiger auftragen, am besten direkt nach dem Duschen auf noch leicht feuchter Haut.
+Für trockene und normale Haut, für Damen und Herren. Nur zur äußerlichen Anwendung. Die Creme enthält ätherisches Geranienöl, bei empfindlicher Haut vor der ersten Anwendung testen.
+Inhalt: 60 ml, Tiegel 5,5 x 5 cm. Inhaltsstoffe (INCI): Aqua, Stearic Acid, Cetyl Alcohol, Simmondsia Chinensis Seed Oil, Isopropyl Myristate, Triethanolamine, Phenoxyethanol, BHT, Pelargonium Graveolens (Geranium) Oil, Allantoin, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Glycerin, Cera Alba, Tocopheryl Acetate, Triticum Vulgare Germ Oil. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>1644</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>bodycream bodybutter gesichtscreme hautpflege feuchtigkeitscreme tagescreme nachtcreme ellbogen reisegröße pflegecreme naturkosmetik handcreme hautcreme pflegemilch nachtpflege tagespflege hydratisierend sensitive geschenkidee muttertag vegan</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>244</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Aqua, Stearic Acid, Cetyl Alcohol, Simmondsia Chinensis Seed Oil, Isopropyl Myristate, Triethanolamine, Phenoxyethanol, BHT, Pelargonium Graveolens (Geranium) Oil, Allantoin, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Glycerin, Cera Alba, Tocopheryl Acetate, Triticum Vulgare Germ Oil</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BF-UJUW-N586</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Rosmarin Haaröl 100 ml mit Rizinusöl und Arganöl</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Ohne Wasser und Silikon, mit Rucolasamen-, Weizenkeim- und Zitronengrasöl, für Kopfhaut und Haarlängen</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Sechs Öle, kein Wasser, kein Silikon: Rizinus-, Rucolasamen-, Weizenkeim- und Arganöl mit ätherischem Rosmarin- und Zitronengrasöl, Sie tragen die reine Ölmischung auf</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Rizinusöl als Basis: Das dickflüssige, klassische Kopfhautöl wird seit Generationen in die Haarwurzeln einmassiert und umhüllt das Haar besser als ein dünnes Öl allein</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Rosmarin und Argan: Rosmarinöl gibt der Mischung den frischen, kräuterigen Duft, Arganöl glättet die Schuppenschicht, damit die Längen glänzen statt nur ölig zu wirken</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Kopfhautmassage: Zwei bis drei Minuten mit den Fingerspitzen einmassieren, so wird die Anwendung zur Routine, die man gern beibehält</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Auch für die Längen: Ein bis zwei Tropfen zwischen den Handflächen verreiben und in trockene Spitzen streichen, so deckt eine Flasche Kopfhautpflege und Finish ab</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>167</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Ein Kopfhaut- und Haaröl aus sechs Ölen und sonst nichts. Es enthält weder Wasser noch Silikon: Auf die Kopfhaut kommt keine verdünnte Lotion, sondern die Ölmischung selbst.
+Rizinusöl bildet die Basis. Es ist das dickflüssige, traditionelle Kopfhautöl, das seit Generationen in die Haarwurzeln einmassiert wird, und es gibt der Mischung genug Substanz, um den Haarschaft zu umhüllen, statt zu verdunsten. Rucolasamenöl und Weizenkeimöl ergänzen es, und Arganöl glättet die Schuppenschicht, sodass das Haar glänzend aussieht.
+Die beiden ätherischen Öle sind Rosmarin und Zitronengras. Rosmarin gibt der Mischung den frischen, kräuterigen Duft, Zitronengras macht ihn spritziger, damit das Öl nicht schwer riecht.
+Anwendung: Das Haar in Partien teilen, entlang jedes Scheitels einige Tropfen auftragen und zwei bis drei Minuten in die Kopfhaut einmassieren. Mindestens eine Stunde einwirken lassen, auf Wunsch auch über Nacht, danach mit Shampoo auswaschen. Für die Längen ein bis zwei Tropfen zwischen den Handflächen verreiben und über trockene Spitzen streichen. Üblich sind ein- bis zweimal pro Woche.
+Geeignet für alle Haartypen, für Damen und Herren. Inhalt: 100 ml, Flasche 13,5 x 4 cm. Inhaltsstoffe (INCI): Ricinus Communis Seed Oil, Eruca Sativa Seed Oil, Triticum Vulgare Germ Oil, Argania Spinosa Kernel Oil, Rosmarinus Officinalis Leaf Oil, Cymbopogon Citratus Oil. Nur zur äußerlichen Anwendung, von Kindern fernhalten. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>1457</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>haarpflege haarserum haarkur haarwuchs haarwachstum pflegeöl ölkur vor haarwäsche spliss damen herren unisex pipette naturkosmetik haarmaske haarbehandlung trockenes geschenk haarpflegeset pflanzenöl</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>203</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Ricinus Communis Seed Oil, Eruca Sativa Seed Oil, Triticum Vulgare Germ Oil, Argania Spinosa Kernel Oil, Rosmarinus Officinalis Leaf Oil, Cymbopogon Citratus Oil</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>YJ-OPSZ-IOCI</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Rosmarin Haarspülung 250 ml mit Argan- und Jojobaöl</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Sulfatfrei, ohne Silikone, Parabene und Mineralöl, mit Weizenkeimöl und Panthenol, entwirrt, für alle Haartypen</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Rosmarin: Der Pflegestoff, nach dem viele suchen, steckt hier in dem Schritt, den Sie nach jeder Haarwäsche ohnehin machen</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Jojoba-, Argan- und Weizenkeimöl: Drei pflegende Pflanzenöle statt Silikon, damit sich das Haar wirklich weicher anfühlt und nicht nur kurz beschichtet</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Leichteres Kämmen: Die Spülung lässt den Kamm durch das nasse Haar gleiten, ohne Ziehen, das an den Spitzen zu Haarbruch führen kann</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Für alle Haartypen: Beschwert feines Haar nicht und pflegt trockene, dicke oder krause Längen, für Damen und Herren, für die ganze Familie</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Passend zum Shampoo: Als Duo mit dem ZAptieka Rosmarin Shampoo konzipiert, funktioniert aber auch mit jedem anderen Shampoo</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Rosmarin ist zum meistbeachteten Inhaltsstoff der Haarpflege geworden, doch die Aufmerksamkeit gilt meist Ölen und Seren. Die Haarspülung wird dabei übersehen, obwohl sie der Schritt ist, den Sie nach jeder einzelnen Haarwäsche verwenden.
+Diese Spülung basiert auf Rosmarin und drei pflegenden Pflanzenölen: Jojoba-, Argan- und Weizenkeimöl. Das ist wichtiger, als es klingt. Viele Spülungen setzen auf Silikone für das Gleitgefühl, das Haar fühlt sich sofort glatt an und nach einer Woche beschichtet. Pflanzenöle pflegen das Haar selbst, sodass die Weichheit auch nach mehreren Haarwäschen bleibt.
+Die Haarspülung ist sulfatfrei und silikonfrei: Sie enthält keine Sulfattenside und keine Silikone, die die Pflege ersetzen.
+Der praktische Vorteil ist das Entwirren. Nach der Wäsche ist das Haar am empfindlichsten, und das Durchziehen des Kamms durch Knoten ist eine häufige Ursache für Haarbruch an den Spitzen. Lässt sich der Kamm frei bewegen, schützt das die Längen über Monate.
+Die Spülung ist für alle Haartypen ausgewogen, für Damen und Herren. Feines Haar wird nicht beschwert, trockene, dicke oder krause Längen werden ausreichend gepflegt. Sie hinterlässt außerdem den kräuterigen Rosmarinduft.
+Anwendung: Nach dem Shampoonieren überschüssiges Wasser ausdrücken, von den Längen bis in die Spitzen auftragen und die Haaransätze aussparen, wenn Ihr Haar schnell fettet. Zwei bis drei Minuten einwirken lassen, durchkämmen und gründlich ausspülen.
+Inhalt: 250 ml, Flasche 19 x 5 cm. Inhaltsstoffe (INCI): Aqua, Cetearyl Alcohol, Cetrimonium Chloride, Glycerin, Simmondsia Chinensis Seed Oil, Triticum Vulgare Germ Oil, Argania Spinosa Kernel Oil, Rosmarinus Officinalis Leaf Oil, Panthenol, Parfum, Methylchloroisothiazolinone, Methylisothiazolinone. Frei von Sulfaten, SLS, SLES, Parabenen, Silikonen und Mineralöl. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>1883</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>conditioner haarkur pflegespülung haarpflege kopfhaut trockenes strapaziertes entwirren kämmbarkeit glanz weich naturkosmetik unisex haarmaske haarbehandlung kopfhautpflege geschenk haarpflegeset rosmarinöl pflanzenöl</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>221</v>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Aqua, Cetearyl Alcohol, Cetrimonium Chloride, Glycerin, Simmondsia Chinensis Seed Oil, Triticum Vulgare Germ Oil, Argania Spinosa Kernel Oil, Rosmarinus Officinalis Leaf Oil, Panthenol, Parfum, Methylchloroisothiazolinone, Methylisothiazolinone</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>308</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="80" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item Name (≤75)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Zeichen</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Item Highlight (≤125)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Zeichen</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet 1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet 2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet 3</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet 4</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet 5</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Max Bullet</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Description (≤2000)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Zeichen</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Search Terms (≤249 Byte)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Byte</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Inhaltsstoffe INCI (TTX)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Gewicht g (TTX)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Hinweis / Compliance</t>
         </is>
       </c>
@@ -2286,11 +2304,11 @@
 Die Basis macht den Unterschied zu einer billigen Seife: Sie besteht aus Sheabutter und Kokosöl, die einen dichten, cremigen Schaum bilden und nach dem Abspülen einen leichten Pflegefilm hinterlassen. Der Duft ist weich und honigartig und stammt aus der Rezeptur selbst, nicht aus einem starken synthetischen Parfüm.
 Die Seife ist für alle Hauttypen ausgewogen und mild genug für die tägliche Anwendung im Gesicht und am Körper.
 Anwendung: Das Stück anfeuchten, in den Händen oder auf einem Luffaschwamm aufschäumen, über Gesicht oder Körper massieren und mit warmem Wasser abspülen. Danach Feuchtigkeitscreme auf die noch leicht feuchte Haut auftragen. Auf einer Seifenschale mit Ablauf aufbewahren, damit das Stück zwischen den Anwendungen trocknet und länger hält.
-Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe: Sodium Palmate, Sodium Palm Kernelate, Aqua, Sheabutter, Kokosöl, Honig, Milch. Geeignet für Gesicht, Körper und Hände. Nur zur äußerlichen Anwendung.</t>
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Mel, Lac. Geeignet für Gesicht, Körper und Hände. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>1382</v>
+        <v>1435</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -2300,7 +2318,15 @@
       <c r="O2" s="2" t="n">
         <v>245</v>
       </c>
-      <c r="P2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Mel, Lac</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2359,11 +2385,11 @@
 Die Basis besteht aus Sheabutter und Kokosöl. Sie sorgen für den dichten, cremigen Schaum und den leichten Pflegefilm nach dem Abspülen, und sie sind der Grund, warum die Seife ohne Sulfattenside gut reinigt.
 Sie ist mild genug für die tägliche Anwendung im Gesicht, am Körper und an den Händen.
 Anwendung: Das Stück anfeuchten, in den Händen oder auf einem Luffaschwamm aufschäumen, über Gesicht oder Körper massieren und mit warmem Wasser abspülen. Danach Feuchtigkeitscreme auf die noch leicht feuchte Haut auftragen. Auf einer Seifenschale mit Ablauf aufbewahren, damit das Stück zwischen den Anwendungen trocknet und länger hält.
-Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe: Sodium Palmate, Sodium Palm Kernelate, Aqua, Sheabutter, Kokosöl, Ziegenmilch (Caprae Lac). Geeignet für Gesicht, Körper und Hände, für trockene und empfindliche Haut, für Damen und Herren. Nur zur äußerlichen Anwendung.</t>
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Caprae Lac. Geeignet für Gesicht, Körper und Hände, für trockene und empfindliche Haut, für Damen und Herren. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>1551</v>
+        <v>1594</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -2373,7 +2399,15 @@
       <c r="O3" s="2" t="n">
         <v>243</v>
       </c>
-      <c r="P3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Caprae Lac</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2431,11 +2465,11 @@
 Sie ist für fettige und Mischhaut gedacht. Das Stück nimmt überschüssiges Öl, Schweiß und Alltagsschmutz auf, doch auf einer Basis aus Sheabutter und Kokosöl, damit die Haut nicht spannt. Diese Balance ist wichtig, denn zu aggressives Waschen bringt fettige Haut dazu, noch mehr Öl zu produzieren.
 Die goldene Farbe stammt von der Kurkuma, nicht von synthetischen Farbstoffen, und der Duft ist die weiche, erdige Note des Gewürzes statt zugesetzten Parfüms. Kurkuma kann helle Waschlappen leicht färben, deshalb den Lappen nach der Anwendung kurz ausspülen.
 Anwendung: Das Stück anfeuchten, in den Händen oder auf einem weichen Waschlappen aufschäumen, etwa 30 Sekunden über das Gesicht massieren und gründlich mit warmem Wasser abspülen. Danach eine leichte Feuchtigkeitscreme auftragen. Am Körper eignet sich die Seife gut für Rücken, Brust und Schultern. Zwischen den Anwendungen auf einer Seifenschale mit Ablauf aufbewahren.
-Für die tägliche Anwendung bei Damen und Herren, auf normaler, Misch- und fetter Haut. Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe: Sodium Palmate, Sodium Palm Kernelate, Aqua, Sheabutter, Kokosöl, Kurkumawurzelpulver (Curcuma Longa). Nur zur äußerlichen Anwendung.</t>
+Für die tägliche Anwendung bei Damen und Herren, auf normaler, Misch- und fetter Haut. Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Curcuma Longa (Turmeric) Root Powder. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1500</v>
+        <v>1575</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -2445,7 +2479,15 @@
       <c r="O4" s="2" t="n">
         <v>243</v>
       </c>
-      <c r="P4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Curcuma Longa (Turmeric) Root Powder</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2504,11 +2546,11 @@
 So lässt sich die Seife leicht täglich verwenden: Sie ist mild genug für normale und trockene Haut, wirksam für Mischhaut, die tagsüber fettig wird, und sanft genug fürs Gesicht, nicht nur unter der Dusche.
 Anwendung: Das Stück anfeuchten, in den Händen oder auf einem Luffaschwamm aufschäumen, über Gesicht oder Körper massieren und mit warmem Wasser abspülen. Danach Feuchtigkeitscreme auf die noch leicht feuchte Haut auftragen. Auf einer Seifenschale mit Ablauf aufbewahren, damit das Stück zwischen den Anwendungen trocknet und länger hält.
 Wer Schwarzkümmelöl bereits als Öl verwendet, bringt mit dieser Seife denselben Inhaltsstoff in den Teil der Routine, der jeden Tag stattfindet.
-Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe: Sodium Palmate, Sodium Palm Kernelate, Aqua, Sheabutter, Kokosöl, Schwarzkümmelöl (Nigella Sativa). Geeignet für Gesicht, Körper und Hände, für Damen und Herren. Nur zur äußerlichen Anwendung.</t>
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Nigella Sativa Seed Oil. Geeignet für Gesicht, Körper und Hände, für Damen und Herren. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1567</v>
+        <v>1632</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -2518,7 +2560,15 @@
       <c r="O5" s="2" t="n">
         <v>244</v>
       </c>
-      <c r="P5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Nigella Sativa Seed Oil</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2577,11 +2627,11 @@
 Darunter liegt eine Basis aus Sheabutter und Kokosöl. Das ist wichtig, denn ein Reiniger, der Öl aggressiv entfernt und die Haut spannen lässt, provoziert nur noch mehr Öl. Hier bleibt die Haut matt und sauber statt strapaziert.
 Die Seife wird in kleinen Chargen von Hand gemacht, kleine Abweichungen zwischen den Stücken sind deshalb normal und kein Mangel. Der Duft ist eine weiche grün-kräuterige Note aus dem Blatt selbst, ohne zugesetztes Parfüm.
 Anwendung: Das Stück anfeuchten, in den Händen oder auf einem weichen Waschlappen aufschäumen, etwa 30 Sekunden über das Gesicht massieren und mit warmem Wasser abspülen. Danach eine leichte Feuchtigkeitscreme auftragen. Auf einer Seifenschale mit Ablauf aufbewahren.
-Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe: Sodium Palmate, Sodium Palm Kernelate, Aqua, Sheabutter, Kokosöl, Sidrblattpulver (Ziziphus Spina-Christi). Nur zur äußerlichen Anwendung.</t>
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Ziziphus Spina-Christi Leaf Powder. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1617</v>
+        <v>1685</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -2591,7 +2641,15 @@
       <c r="O6" s="2" t="n">
         <v>241</v>
       </c>
-      <c r="P6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Ziziphus Spina-Christi Leaf Powder</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2650,11 +2708,11 @@
 Für viele Männer ist sie die Standardseife, weil sie alles auf einmal erledigt: kein Parfüm, keine komplizierte Routine, ein schwarzes Stück für Gesicht, Körper und Hände.
 Die Farbe stammt von der Kohle, nicht von synthetischen Farbstoffen. Deshalb schäumt sie in den ersten Sekunden dunkel, und es lohnt sich, Waschlappen oder Luffa nach der Anwendung auszuspülen.
 Anwendung: Das Stück anfeuchten, in den Händen oder auf einem Luffaschwamm aufschäumen, etwa 30 Sekunden über das Gesicht massieren und gründlich mit warmem Wasser abspülen. Danach Feuchtigkeitscreme auftragen, besonders bei Mischhaut. Auf einer Seifenschale mit Ablauf aufbewahren.
-Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe: Sodium Palmate, Sodium Palm Kernelate, Aqua, Sheabutter, Kokosöl, Kohlepulver. Geeignet für die tägliche Anwendung an Gesicht, Körper und Händen. Nur zur äußerlichen Anwendung.</t>
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Charcoal Powder. Geeignet für die tägliche Anwendung an Gesicht, Körper und Händen. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1502</v>
+        <v>1580</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -2664,7 +2722,15 @@
       <c r="O7" s="2" t="n">
         <v>238</v>
       </c>
-      <c r="P7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii (Shea) Butter, Cocos Nucifera (Coconut) Oil, Charcoal Powder</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2723,12 +2789,12 @@
 Die übrige Inhaltsstoffliste ist kurz, und jeder Bestandteil hat eine Aufgabe. Sesam-, Jojoba- und Olivenöl tragen das Zinkoxid, damit es sich gleichmäßig verteilt und nicht streift, und sie halten die Haut geschmeidig, statt sie an einem Tag in der Sonne auszutrocknen. Lavendelöl gibt der Lotion ihren Duft.
 Mineralische Sonnencreme gilt als dick, weißelnd und schwer einzureiben, deshalb tragen viele zu wenig auf. Diese Lotion ist bewusst leicht: Sie verteilt sich gut, zieht ein und fühlt sich angenehm statt klebrig an, sodass ein großzügiges, korrektes Auftragen realistisch ist.
 Anwendung: Großzügig auf saubere, trockene Haut auftragen, 15 bis 30 Minuten bevor Sie in die Sonne gehen. Für den ganzen Körper eines Erwachsenen sind etwa sechs bis acht Teelöffel nötig. Mindestens alle zwei Stunden erneut auftragen, und immer nach dem Schwimmen, starkem Schwitzen oder Abtrocknen mit dem Handtuch.
-Meiden Sie die Sonne zwischen 11 und 15 Uhr, schützen Sie sich mit Kleidung und Hut und halten Sie Babys und kleine Kinder aus der direkten Sonne fern. Übermäßige Sonnenbestrahlung ist ein ernstes Gesundheitsrisiko.
-Inhalt: 125 ml, Flasche 12,5 x 4 cm. Inhaltsstoffe: Sesamsamenöl, Zinkoxid, Jojobasamenöl, Olivenöl, Lavendelöl. Nur zur äußerlichen Anwendung, Augenkontakt vermeiden, nicht auf verletzte oder gereizte Haut auftragen.</t>
+Meiden Sie die Mittagssonne, schützen Sie sich mit Kleidung und Hut und halten Sie Babys aus der direkten Sonne fern. Übermäßige Sonnenbestrahlung ist ein ernstes Gesundheitsrisiko.
+Inhalt: 125 ml, Flasche 12,5 x 4 cm. Inhaltsstoffe (INCI): Sesamum Indicum (Sesame) Seed Oil, Zinc Oxide, Simmondsia Chinensis (Jojoba) Seed Oil, Olea Europaea (Olive) Fruit Oil, Lavandula Angustifolia (Lavender) Oil. Nur zur äußerlichen Anwendung, Augenkontakt vermeiden, nicht auf verletzte oder gereizte Haut auftragen. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1886</v>
+        <v>1979</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -2738,7 +2804,15 @@
       <c r="O8" s="2" t="n">
         <v>164</v>
       </c>
-      <c r="P8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Sesamum Indicum (Sesame) Seed Oil, Zinc Oxide, Simmondsia Chinensis (Jojoba) Seed Oil, Olea Europaea (Olive) Fruit Oil, Lavandula Angustifolia (Lavender) Oil</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2798,11 +2872,11 @@
 Es ist unraffiniert und lösungsmittelfrei. Es gibt keine Hitzeraffination, keine chemische Extraktion und keine Streckung mit billigeren Trägerölen, und deshalb schmeckt es kräftig. Wer ein mildes Öl erwartet, ist beim ersten Mal meist überrascht.
 Verwendung: Schwarzkümmelöl wird traditionell teelöffelweise eingenommen, pur oder mit Honig, und kommt auch in Speisen und in Ölmischungen für Haar und Kopfhaut zum Einsatz. Wenn Sie es noch nicht kennen, beginnen Sie mit einer kleinen Menge, denn der Geschmack ist intensiv.
 Kühl und dunkel mit geschlossenem Deckel lagern. Die Braunglasflasche schützt das Öl vor Licht.
-Inhalt: 100 ml, Flasche 13 x 5 cm aus Braunglas. Einzige Zutat: 100 Prozent Nigella-Sativa-Samenöl, erste Kaltpressung, unraffiniert.</t>
+Inhalt: 100 ml, Flasche 13 x 5 cm aus Braunglas. Inhaltsstoffe (INCI): Nigella Sativa Seed Oil. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1555</v>
+        <v>1539</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -2813,6 +2887,14 @@
         <v>122</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Nigella Sativa Seed Oil</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>LEBENSMITTEL: DE-Etikett nach LMIV (Zutatenverzeichnis, MHD, Nährwerttabelle, verantwortlicher Lebensmittelunternehmer in der EU) prüfen; keine gesundheitsbezogenen Aussagen.</t>
         </is>
@@ -2875,11 +2957,11 @@
 Es gibt zwei übliche Verwendungen. In der Küche gilt es als kräftiges Finishing-Öl und wird traditionell in kleinen Mengen eingenommen. Für das Haar ist es eines der klassischen Öle zur Haarölpflege: leicht erwärmt in Kopfhaut und Längen massiert, eine Stunde oder über Nacht einwirken lassen und vor dem Waschen mit Shampoo auswaschen.
 Anwendung fürs Haar: Eine kleine Menge in den Handflächen erwärmen, in die Kopfhaut einmassieren und durch die Längen ziehen, mindestens eine Stunde einwirken lassen und auswaschen. Für Speisen: einen Teelöffel auf einmal, der Geschmack ist kräftig.
 Kühl und dunkel mit geschlossenem Deckel lagern.
-Inhalt: 100 ml, Flasche 13 x 5 cm aus Braunglas. Einzige Zutat: 100 Prozent Eruca-Sativa-Samenöl, kaltgepresst, unraffiniert.</t>
+Inhalt: 100 ml, Flasche 13 x 5 cm aus Braunglas. Inhaltsstoffe (INCI): Eruca Sativa Seed Oil. Haltbarkeit: 2 Jahre.</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1419</v>
+        <v>1409</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2891,7 +2973,463 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
+          <t>Eruca Sativa Seed Oil</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
           <t>STOPP: Rucolasamenöl (Eruca sativa) enthält typischerweise sehr viel Erucasäure. In der EU gelten Höchstgehalte für Erucasäure in Lebensmitteln (VO (EU) 2019/1870); Laborwert (Erucasäure) und Verkehrsfähigkeit als Lebensmittel in DE vor Listing klären. Bis dahin NICHT veröffentlichen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2L-CFOT-WAF5</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Kamelmilchseife 100 g für Gesicht und Körper</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Stückseife mit Sheabutter und Kokosöl, milde Reinigung für trockene und empfindliche Haut, unparfümiert</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Echte Kamelmilch: Im Nahen Osten seit Jahrhunderten in der Hautpflege verwendet, bringt von Natur aus Proteine, Vitamine und Fette in die Seife</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Sheabutter und Kokosöl: Pflanzenbutter und Öle statt billiger Füllstoffe, für guten Schaum und ein weiches, angenehmes Hautgefühl nach dem Abspülen</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Für trockene und empfindliche Haut: Milde Rezeptur ohne starken Duft, geeignet für Haut, die auf stark parfümierte Duschgele reagiert, für Gesicht und Körper</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Ohne SLS, ohne künstliche Farbstoffe: Hergestellt ohne Sulfattenside, synthetische Farbstoffe und aggressive Tenside, das macht den Unterschied zur austrocknenden Seife</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Ein Stück statt Plastikflasche: 100 g halten bei täglicher Nutzung lange und kommen ohne Pumpspender aus, ein einfacher Tausch fürs plastikärmere Bad</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Ein Reinigungsstück rund um Kamelmilch, einen Inhaltsstoff, der im Nahen Osten in der Hautpflege verwendet wurde, lange bevor es moderne Kosmetik gab. Kamelmilch enthält von Natur aus Proteine, Milchfette und Vitamine. In einer Seife bedeutet das etwas Einfaches und Spürbares: Die Haut fühlt sich nach dem Waschen angenehm an statt gespannt und quietschend.
+Auch der Rest der Rezeptur zählt. Die Seife basiert auf Sheabutter und Kokosöl, die einen guten Schaum erzeugen und nach dem Abspülen ein weiches Hautgefühl hinterlassen. Sie ist ohne Sulfattenside und ohne künstliche Farbstoffe hergestellt.
+Die Seife ist für alle Hauttypen gedacht, besonders für trockene und empfindliche Haut, und mild genug für Gesicht und Körper.
+Anwendung: Das Stück anfeuchten, in den Händen oder auf einem Luffaschwamm aufschäumen, über Gesicht oder Körper massieren und mit warmem Wasser abspülen. Danach Feuchtigkeitscreme auf die noch leicht feuchte Haut auftragen. Auf einer Seifenschale mit Ablauf aufbewahren, damit das Stück zwischen den Anwendungen trocknet und länger hält.
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Camelus Dromedarius Milk. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>1308</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>naturseife handseife gesichtsseife körperseife seifenstück duschseife feste damen herren unisex geschenk reisen milchseife sensitive seifenschale reisebegleiter geschenkidee badezimmer handgemacht naturkosmetik pflanzenöle körperpflege</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>239</v>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Camelus Dromedarius Milk</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>WJ-9EH3-NUHN</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Weihrauch Seife 100 g für Gesicht und Körper</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Stückseife mit Boswellia, Sheabutter und Kokosöl, milde tägliche Reinigung für alle Hauttypen, ohne Sulfate</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Mit Weihrauch: Boswellia wird seit Jahrtausenden in Hautritualen verwendet und gibt der Seife einen warmen, harzigen Duft, ganz anders als Frucht- und Blumenseifen</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Mild fürs Gesicht: Reinigt das Gesicht, ohne es auszutrocknen, deshalb morgens und abends nutzbar und nicht nur unter der Dusche</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Sheabutter und Kokosöl: Pflanzenbutter und Öl sorgen für cremigen Schaum und ein gepflegtes Hautgefühl statt der Spannung einer Detergenzienseife</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Für alle Hauttypen: Ausgewogen für normale, trockene und Mischhaut und frei von aggressiven Sulfaten, sodass die ganze Familie ein Stück teilen kann</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Ein Duft zum Behalten: Die natürliche Weihrauchnote ist warm und leicht rauchig und stammt aus dem ätherischen Öl statt aus synthetischem Parfüm</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Weihrauch ist das Harz des Boswellia-Baums und wird seit Jahrtausenden in Hautritualen und Zeremonien verwendet. In einer Seife fällt sofort der warme, harzige und leicht rauchige Duft auf, der sich deutlich von den Frucht- und Blumenseifen der meisten Regale unterscheidet.
+Die Rezeptur ist bewusst einfach gehalten. Sheabutter und Kokosöl bilden die Basis, erzeugen einen dichten, cremigen Schaum und lassen die Haut nach dem Abspülen weich zurück, statt sie wie eine Detergenzienseife zu spannen. Ätherisches Weihrauchöl gibt den Duft.
+Die Seife ist für alle Hauttypen ausgewogen, mild genug für die tägliche Gesichtsreinigung und frei von aggressiven Sulfaten.
+Anwendung: Das Stück anfeuchten, in den Händen oder auf einem Luffaschwamm aufschäumen, über Gesicht oder Körper massieren und mit warmem Wasser abspülen. Danach Feuchtigkeitscreme auf die noch leicht feuchte Haut auftragen. Auf einer Seifenschale mit Ablauf aufbewahren, damit das Stück zwischen den Anwendungen trocknet und länger hält.
+Gewicht: 100 g, Stückgröße 8 x 5 x 2,5 cm. Inhaltsstoffe (INCI): Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Boswellia Carterii Oil. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>1243</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>naturseife handseife gesichtsseife körperseife seifenstück duschseife feste damen herren unisex geschenk reisen olibanum frankincense seifenschale reisebegleiter geschenkidee badezimmer handgemacht naturkosmetik pflanzenöle körperpflege</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Sodium Palmate, Sodium Palm Kernelate, Aqua, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Boswellia Carterii Oil</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>N4-FRNJ-Q53V</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Nachtcreme 60 ml mit Kurkuma und Orange für das Gesicht</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Mit Sheabutter und Pflanzenölen, Feuchtigkeitspflege über Nacht, für normale, trockene und Mischhaut</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Für die Nacht gemacht: Nachts darf eine Creme reichhaltiger sein, denn nichts muss unter Make-up sitzen, deshalb ist die Rezeptur großzügiger als bei einer Tagescreme</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Kurkuma: Curcuma Longa ist der Inhaltsstoff, den viele für ihre Pflegeroutine suchen, und gibt der Creme ihre warme goldene Farbe ganz ohne synthetische Farbstoffe</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Orangenöl: Eine weiche Zitrusnote hebt die erdige Kurkuma an und macht die Creme zum angenehmen letzten Schritt vor dem Schlafengehen</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Sheabutter und Pflanzenöle: Die Basis pflegt die Haut über Nacht, damit sie sich morgens weich und angenehm anfühlt statt gespannt</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Reichhaltig, aber nicht schwer: Zieht ein, bevor Sie sich hinlegen, statt auf den Kopfkissenbezug überzugehen</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>166</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Eine Nachtcreme darf reichhaltiger sein als eine Tagescreme, weil nichts unter Make-up liegen muss und die Haut acht ungestörte Stunden zum Aufnehmen hat. Diese Creme nutzt genau das.
+Kurkuma ist der Inhaltsstoff, den viele für ihre Pflegeroutine suchen. Curcuma Longa gibt der Creme ihre warme goldene Farbe auf natürliche Weise, ohne synthetische Farbstoffe. Das ätherische Orangenöl hebt die erdige Note der Kurkuma mit einem weichen Zitrusduft an.
+Die Basis aus Sheabutter und Pflanzenölen pflegt die Haut durch die Nacht. Die Creme ist reichhaltig, aber nicht schwer, und zieht ein, bevor Sie sich hinlegen.
+Anwendung: Abends auf die gereinigte Haut von Gesicht und Hals auftragen. Eine kleine Menge zwischen den Fingerspitzen erwärmen und sanft einarbeiten. Für normale, trockene und Mischhaut. Inhalt: 60 ml, Tiegel 5,5 x 5 cm. Inhaltsstoffe (INCI): Aqua, Stearic Acid, Cetyl Alcohol, Simmondsia Chinensis Seed Oil, Isopropyl Myristate, Triethanolamine, Phenoxyethanol, BHT, Citrus Aurantium Dulcis Peel Oil, Allantoin, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Glycerin, Cera Alba, Tocopheryl Acetate, Triticum Vulgare Germ Oil, Curcuma Longa (Turmeric) Extract. Nur zur äußerlichen Anwendung. Haltbarkeit: 2 Jahre.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>1238</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>nachtpflege gesichtscreme gelbwurz kurkumacreme pflegecreme hautpflege damen herren unisex naturkosmetik bodybutter handcreme hautcreme pflegemilch tagespflege hydratisierend sensitive geschenkidee weihnachtsgeschenk muttertag vegan</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>232</v>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Aqua, Stearic Acid, Cetyl Alcohol, Simmondsia Chinensis Seed Oil, Isopropyl Myristate, Triethanolamine, Phenoxyethanol, BHT, Citrus Aurantium Dulcis Peel Oil, Allantoin, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Glycerin, Cera Alba, Tocopheryl Acetate, Triticum Vulgare Germ Oil, Curcuma Longa (Turmeric) Extract</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Passt in den vorhandenen DE-Feed (SKIN_MOISTURIZER). Auf UK Inactive, daher nicht im Feed enthalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>R1-RAXF-Z5I9</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ZAptieka Weihrauch Hydrolat 100 ml, Gesichtswasser und Gesichtsspray</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Dampfdestilliert aus Boswellia-Harz, alkoholfrei, Toner und Face Mist in einem, für alle Hauttypen</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Echtes dampfdestilliertes Hydrolat: Weihrauchwasser, das bei der Dampfdestillation von Boswellia-Harz entsteht, mit nur einem leichten Konservierungssystem, kein parfümiertes Wasser</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Alkoholfrei: Viele klassische Toner arbeiten mit Alkohol und lassen die Haut spannen, dieses erfrischt und spendet Feuchtigkeit und eignet sich für mehrmals täglich</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Toner und Gesichtsspray in einem: Nach der Reinigung mit dem Wattepad auftragen, um die Haut auf die Pflege vorzubereiten, oder tagsüber direkt auf das Gesicht sprühen</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Wie Rosenwasser, nur anders: Ein Hydrolat entsteht wie Rosenwasser durch Dampfdestillation der Pflanze, dieses aus Weihrauchharz duftet warm und harzig statt blumig</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Warmer harziger Duft: Das Aroma stammt nur vom Weihrauch selbst, ohne zugesetztes Parfüm, das unterscheidet ein echtes Hydrolat von einem parfümierten Wasser</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Ein Hydrolat bleibt zurück, nachdem eine Pflanze dampfdestilliert wurde: das aromatische Wasser, das den Duft und den wasserlöslichen Teil der Pflanze trägt. Dieses hier ist Weihrauchwasser, destilliert aus Boswellia-Harz. Außerdem enthält die Flasche nur die kleinen Mengen Natriumbenzoat, Kaliumsorbat und Zitronensäure, die nötig sind, um ein Produkt auf Wasserbasis nach dem Öffnen haltbar zu machen.
+Diese Schlichtheit ist der Punkt. Das Hydrolat ist alkoholfrei, riecht warm und harzig und lässt sich als Gesichtswasser nach der Reinigung wie auch als Gesichtsspray über den Tag und über Make-up verwenden.
+Anwendung: Nach der Reinigung mit einem Wattepad über das Gesicht streichen oder aus etwa 20 cm Abstand aufsprühen, danach die Pflege auftragen. Für alle Hauttypen.
+Aufbewahrung: Zum Erhalt der Eigenschaften kühl und dunkel lagern, am besten im Kühlschrank. Da keine aggressiven Konservierungsmittel verwendet werden, nach dem Öffnen innerhalb von 6 bis 12 Monaten aufbrauchen. Vor der ersten Anwendung an einer kleinen Hautstelle testen. Augenkontakt vermeiden. Nur zur äußerlichen Anwendung.
+Inhalt: 100 ml, Flasche 14 x 4 cm. Inhaltsstoffe (INCI): Boswellia Carterii Resin Extract, Sodium Benzoate, Potassium Sorbate, Citric Acid.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>facemist olibanum carterii naturkosmetik pflegespray erfrischung damen herren unisex geschenk naturprodukt</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Boswellia Carterii Resin Extract, Sodium Benzoate, Potassium Sorbate, Citric Acid</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Anderer Produkttyp (ASTRINGENT_SUBSTANCE). Auf UK Inactive. Aus der Beschreibung der TTX-Tabelle (Lifting, Falten, Entzündungen, Haare) wurde nichts übernommen: Stufe-1-Aussagen.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Product type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Template nötig</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SKIN_CLEANING_AGENT (Seife)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>79-IMQK-CFL6, AL-OBXA-2JAB, BO-LDT0-9J23, O7-OU4A-2PTM, RY-63EN-QQ04, SO-33NV-Y8TE (+ inactive: 2L-CFOT-WAF5, WJ-9EH3-NUHN)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SUNSCREEN (Sonnenschutz)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>B8-S7B1-XUBY</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>EDIBLE_OIL_VEGETABLE (Speiseöl)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>GO-HRO6-WM8V (H3-5FMC-FAD4 erst nach Compliance-Prüfung)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ASTRINGENT_SUBSTANCE (Gesichtswasser)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>R1-RAXF-Z5I9 (inactive)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nur falls gewünscht</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SKIN_MOISTURIZER, SHAMPOO</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>bereits im DE-Template, Feed fertig</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final DE upload feed: 19 SKUs (incl. H3), EUR=GBP*1.19, qty 2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDVF22cVHqURRrq6mrUjqS
</commit_message>
<xml_diff>
--- a/DE_Feed_Missing_Positions/DE_SEO_Texte_Missing_Positions.xlsx
+++ b/DE_Feed_Missing_Positions/DE_SEO_Texte_Missing_Positions.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>DE price EUR (UK x 1.1557)</t>
+          <t>DE price EUR (UK x 1.19)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -522,7 +522,7 @@
         <v>27.99</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>32.35</v>
+        <v>33.31</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         <v>54.99</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>63.55</v>
+        <v>65.44</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -608,7 +608,7 @@
         <v>52.99</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>61.24</v>
+        <v>63.06</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -651,16 +651,16 @@
         <v>19.99</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>23.1</v>
+        <v>23.79</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Тип SKIN_CLEANING_AGENT отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SKIN_CLEANING_AGENT, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -694,16 +694,16 @@
         <v>19.99</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>23.1</v>
+        <v>23.79</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Тип SKIN_CLEANING_AGENT отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SKIN_CLEANING_AGENT, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -737,16 +737,16 @@
         <v>29.99</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>34.66</v>
+        <v>35.69</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Тип SUNSCREEN отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SUNSCREEN, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
         <v>45.99</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>53.15</v>
+        <v>54.73</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -823,16 +823,16 @@
         <v>19.99</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>23.1</v>
+        <v>23.79</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Тип SKIN_CLEANING_AGENT отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SKIN_CLEANING_AGENT, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
         <v>25.99</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>30.04</v>
+        <v>30.93</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v>35.99</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>41.59</v>
+        <v>42.83</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -952,16 +952,16 @@
         <v>29.99</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>34.66</v>
+        <v>35.69</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Тип EDIBLE_OIL_VEGETABLE отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип EDIBLE_OIL_VEGETABLE, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -995,16 +995,16 @@
         <v>29.99</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>34.66</v>
+        <v>35.69</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>СТОП: проверка комплаенса</t>
+          <t>В фиде (решение владельца)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Erucasäure-Grenzwerte (VO (EU) 2019/1870), см. README</t>
+          <t>Сертификаты у владельца, загрузить в Account Health; Erucasäure-Grenzwerte (VO (EU) 2019/1870) см. README</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
         <v>52.99</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>61.24</v>
+        <v>63.06</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1081,16 +1081,16 @@
         <v>19.99</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>23.1</v>
+        <v>23.79</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Тип SKIN_CLEANING_AGENT отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SKIN_CLEANING_AGENT, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -1124,16 +1124,16 @@
         <v>19.99</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>23.1</v>
+        <v>23.79</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Тип SKIN_CLEANING_AGENT отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SKIN_CLEANING_AGENT, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -1167,16 +1167,16 @@
         <v>19.99</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>23.1</v>
+        <v>23.79</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, нужен другой шаблон DE</t>
+          <t>В фиде</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Тип SKIN_CLEANING_AGENT отсутствует в загруженном DE-шаблоне</t>
+          <t>Тип SKIN_CLEANING_AGENT, шаблон DEUTSCH ..._SKIN_MOISTURIZER.xlsm</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
         <v>27.99</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>32.35</v>
+        <v>33.31</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         <v>35.99</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>41.59</v>
+        <v>42.83</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
         <v>27.99</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>32.35</v>
+        <v>33.31</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         <v>28.99</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>33.5</v>
+        <v>34.5</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1382,16 +1382,16 @@
         <v>11.99</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>13.86</v>
+        <v>14.27</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, Inactive на UK</t>
+          <t>В фиде (Inactive на UK)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
+          <t>Включён по решению владельца</t>
         </is>
       </c>
     </row>
@@ -1425,16 +1425,16 @@
         <v>24.99</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>28.88</v>
+        <v>29.74</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, Inactive на UK</t>
+          <t>В фиде (Inactive на UK)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
+          <t>Включён по решению владельца</t>
         </is>
       </c>
     </row>
@@ -1468,16 +1468,16 @@
         <v>21.99</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>25.41</v>
+        <v>26.17</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, Inactive на UK</t>
+          <t>В фиде (Inactive на UK)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
+          <t>Включён по решению владельца</t>
         </is>
       </c>
     </row>
@@ -1511,16 +1511,16 @@
         <v>11.99</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>13.86</v>
+        <v>14.27</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Тексты готовы, Inactive на UK</t>
+          <t>В фиде (Inactive на UK)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Не в фиде: листинг на UK неактивен, решение за владельцем</t>
+          <t>Включён по решению владельца</t>
         </is>
       </c>
     </row>

</xml_diff>